<commit_message>
update dummy data for testing
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/dummy_data_example_network.xlsx
+++ b/01_data/01_input_data/02_processed/dummy_data_example_network.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55117D7A-CA19-450C-A274-70359ECA6554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A0B7B9-DC7E-42CB-8D9F-90509D1A38E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -802,6 +802,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
   <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="3" width="14.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1307,10 +1310,10 @@
         <v>23</v>
       </c>
       <c r="D18">
-        <v>3.852038590666667</v>
+        <v>30</v>
       </c>
       <c r="E18">
-        <v>3.852038590666667</v>
+        <v>30</v>
       </c>
       <c r="F18">
         <v>6</v>
@@ -2025,7 +2028,7 @@
         <v>15</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -2047,7 +2050,7 @@
         <v>17</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add plot for mapping demand and resolve data issue
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/dummy_data_example_network.xlsx
+++ b/01_data/01_input_data/02_processed/dummy_data_example_network.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/mar_eco_cbs_dk/Documents/Desktop/hydrogen_grid/01_data/01_input_data/02_processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A0B7B9-DC7E-42CB-8D9F-90509D1A38E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{29A0B7B9-DC7E-42CB-8D9F-90509D1A38E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12C26F7C-B195-4445-8D2A-FEC04A55F69F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="33">
   <si>
     <t>Commodities</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>node_0008_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -194,6 +197,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -800,13 +807,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="3" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -835,7 +842,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -864,7 +871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -893,7 +900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -922,7 +929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -951,7 +958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -980,7 +987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1009,7 +1016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1038,7 +1045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1067,7 +1074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1096,7 +1103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1125,7 +1132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1154,7 +1161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1183,7 +1190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1211,8 +1218,11 @@
       <c r="I14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="M14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1241,7 +1251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>11</v>
       </c>

</xml_diff>